<commit_message>
2026-09-09 19:33 AldlistPM Upd
</commit_message>
<xml_diff>
--- a/PM/SkienAlgsListPM2025.xlsx
+++ b/PM/SkienAlgsListPM2025.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://urfume-my.sharepoint.com/personal/sergey_osipov_urfu_me/Documents/AiSD2026/PM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1297" documentId="13_ncr:1_{BB64072A-02B6-4C3F-B1E2-71C6B558E3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35BC7EB5-76C1-4E73-B4C1-35E98C180939}"/>
+  <xr:revisionPtr revIDLastSave="1301" documentId="13_ncr:1_{BB64072A-02B6-4C3F-B1E2-71C6B558E3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA9C9442-ACDF-476C-A7A3-5E4694D2915B}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="660" windowWidth="24660" windowHeight="14640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="105" yWindow="750" windowWidth="24660" windowHeight="14640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="324">
   <si>
     <t>Листинг</t>
   </si>
@@ -1030,6 +1031,9 @@
   </si>
   <si>
     <t>Бельков Сергей Дмитриевич</t>
+  </si>
+  <si>
+    <t>Гультяева Виктория Юрьевна</t>
   </si>
 </sst>
 </file>
@@ -1709,7 +1713,7 @@
       </c>
       <c r="G2" s="14"/>
       <c r="H2" s="3" t="str" cm="1">
-        <f t="array" ref="H2:H9">_xlfn.UNIQUE($F$2:$F$107)</f>
+        <f t="array" ref="H2:H10">_xlfn.UNIQUE($F$2:$F$107)</f>
         <v>Толстобров Дмитрий Александрович</v>
       </c>
       <c r="I2" s="4">
@@ -1870,11 +1874,11 @@
       <c r="F8" s="11"/>
       <c r="G8" s="17"/>
       <c r="H8" s="3" t="str">
-        <v>Бельков Сергей Дмитриевич</v>
+        <v>Гультяева Виктория Юрьевна</v>
       </c>
       <c r="I8" s="4">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1896,11 +1900,11 @@
       <c r="F9" s="11"/>
       <c r="G9" s="17"/>
       <c r="H9" s="5" t="str">
-        <v>Корнешов Дмитрий Александрович</v>
+        <v>Бельков Сергей Дмитриевич</v>
       </c>
       <c r="I9" s="4">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1921,10 +1925,12 @@
       </c>
       <c r="F10" s="11"/>
       <c r="G10" s="17"/>
-      <c r="H10" s="3"/>
+      <c r="H10" s="3" t="str">
+        <v>Корнешов Дмитрий Александрович</v>
+      </c>
       <c r="I10" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2525,7 +2531,9 @@
       <c r="E34" s="3">
         <v>12</v>
       </c>
-      <c r="F34" s="11"/>
+      <c r="F34" s="8" t="s">
+        <v>323</v>
+      </c>
       <c r="G34" s="14"/>
       <c r="H34" s="3"/>
       <c r="I34" s="4">
@@ -2549,7 +2557,9 @@
       <c r="E35" s="3">
         <v>11</v>
       </c>
-      <c r="F35" s="11"/>
+      <c r="F35" s="8" t="s">
+        <v>323</v>
+      </c>
       <c r="G35" s="19"/>
       <c r="H35" s="5"/>
       <c r="I35" s="4">
@@ -2573,7 +2583,9 @@
       <c r="E36" s="3">
         <v>14</v>
       </c>
-      <c r="F36" s="12"/>
+      <c r="F36" s="8" t="s">
+        <v>323</v>
+      </c>
       <c r="G36" s="14"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4">

</xml_diff>